<commit_message>
change(preview): video chỉ hiện link YouTube nếu đã upload, bỏ mp4 cục bộ
Trước đó preview hiện poster + ghi chú cho mọi file mp4 cục bộ. Giờ:
- KHÔNG đụng file mp4 cục bộ nữa.
- Đọc youtube_url từ Sheet Result. Có → hiện nút "▶ Xem video trên YouTube" + link.
  Chưa upload YouTube → không đính kèm video gì cả.

Preview vẫn tự chứa: ảnh + audio nhúng base64, video chỉ là href link (vốn phải online).
Bỏ tham số --embed-video. Cập nhật AGENTS + workflow index.

UAT 2 case: TOBI-001 (có youtube_url) → hiện link; TOBI-002 (chưa upload) → 0 nhắc video.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0118F3Rvc799gvJE5ZsHAsH7
</commit_message>
<xml_diff>
--- a/content/KPIM/02_campaigns/01_Tobi_Posts/01_Tobi_Posts.xlsx
+++ b/content/KPIM/02_campaigns/01_Tobi_Posts/01_Tobi_Posts.xlsx
@@ -1138,7 +1138,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1190,6 +1190,43 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TOBI-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://ducnguyen.vn/atlas/ai/ai-agent-la-gi</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://youtu.be/DEMO-001</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>100_123</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://facebook.com/DEMO-001</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>published</t>
         </is>
       </c>
     </row>

</xml_diff>